<commit_message>
docs: insertar logo del SENA en el encabezado de la guía de autoevaluación
</commit_message>
<xml_diff>
--- a/Guia_Autoevaluacion_Frontend_Diligenciada.xlsx
+++ b/Guia_Autoevaluacion_Frontend_Diligenciada.xlsx
@@ -724,6 +724,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="561975" cy="552450"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4268,6 +4298,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="48" min="0" max="16383" man="1"/>
   </rowBreaks>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>